<commit_message>
added in traders (3 and 5)
</commit_message>
<xml_diff>
--- a/Historical Excel/Round 3/Trades Day 0 (Round 3).xlsx
+++ b/Historical Excel/Round 3/Trades Day 0 (Round 3).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/92c4f7ffed9c6980/Python/IntaraTradingAlgorithm/Historical Excel/Round 3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="8_{7202C9AC-DBDA-4DAE-A655-BBAB2AB1A8DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2665D8EF-9BF6-4EC2-A722-2B2B0E644EA1}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="8_{7202C9AC-DBDA-4DAE-A655-BBAB2AB1A8DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02D0EEC7-5EEC-43DE-A463-C36CD52E0DAD}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{541F6641-1DF7-4112-B6A0-82C8F2B62C88}"/>
   </bookViews>
@@ -6535,15 +6535,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>327025</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:colOff>364378</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>94503</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>22225</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>476250</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>75452</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -6961,7 +6961,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF09FFBA-DC5C-4F1B-AAD7-54D3429170B0}">
-  <dimension ref="A1:G1309"/>
+  <dimension ref="A1:J1309"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.1796875" bestFit="1" customWidth="1"/>
@@ -14333,7 +14333,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="321" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A321">
         <v>977200</v>
       </c>
@@ -14356,7 +14356,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="322" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A322">
         <v>980400</v>
       </c>
@@ -14379,7 +14379,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="323" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A323">
         <v>990400</v>
       </c>
@@ -14402,7 +14402,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="324" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A324">
         <v>997000</v>
       </c>
@@ -14425,7 +14425,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="325" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A325">
         <v>999900</v>
       </c>
@@ -14448,7 +14448,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="326" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A326">
         <v>2500</v>
       </c>
@@ -14470,8 +14470,12 @@
       <c r="G326">
         <v>4</v>
       </c>
-    </row>
-    <row r="327" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="J326">
+        <f>AVERAGE(F326:F770)</f>
+        <v>5246.0808988764047</v>
+      </c>
+    </row>
+    <row r="327" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A327">
         <v>5200</v>
       </c>
@@ -14494,7 +14498,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="328" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A328">
         <v>5500</v>
       </c>
@@ -14517,7 +14521,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="329" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A329">
         <v>9300</v>
       </c>
@@ -14540,7 +14544,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="330" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A330">
         <v>11900</v>
       </c>
@@ -14563,7 +14567,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="331" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A331">
         <v>14000</v>
       </c>
@@ -14586,7 +14590,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="332" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A332">
         <v>17000</v>
       </c>
@@ -14609,7 +14613,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="333" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A333">
         <v>19900</v>
       </c>
@@ -14632,7 +14636,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="334" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A334">
         <v>20700</v>
       </c>
@@ -14655,7 +14659,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="335" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A335">
         <v>22500</v>
       </c>
@@ -14678,7 +14682,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="336" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A336">
         <v>23200</v>
       </c>

</xml_diff>

<commit_message>
uploads (3 is best, 4 is good)
</commit_message>
<xml_diff>
--- a/Historical Excel/Round 3/Trades Day 0 (Round 3).xlsx
+++ b/Historical Excel/Round 3/Trades Day 0 (Round 3).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/92c4f7ffed9c6980/Python/IntaraTradingAlgorithm/Historical Excel/Round 3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="8_{7202C9AC-DBDA-4DAE-A655-BBAB2AB1A8DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02D0EEC7-5EEC-43DE-A463-C36CD52E0DAD}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="8_{7202C9AC-DBDA-4DAE-A655-BBAB2AB1A8DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FDE01822-2EF7-421F-9D16-BB689F322235}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{541F6641-1DF7-4112-B6A0-82C8F2B62C88}"/>
   </bookViews>
@@ -6973,7 +6973,7 @@
     <col min="7" max="7" width="10.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -6996,7 +6996,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>8000</v>
       </c>
@@ -7019,7 +7019,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>10100</v>
       </c>
@@ -7042,7 +7042,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>15300</v>
       </c>
@@ -7065,7 +7065,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>15700</v>
       </c>
@@ -7087,8 +7087,12 @@
       <c r="G5">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="J5">
+        <f>AVERAGE(F2:F325)</f>
+        <v>9990.5493827160499</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>16400</v>
       </c>
@@ -7111,7 +7115,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>20300</v>
       </c>
@@ -7134,7 +7138,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>20500</v>
       </c>
@@ -7157,7 +7161,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>23300</v>
       </c>
@@ -7180,7 +7184,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>28500</v>
       </c>
@@ -7203,7 +7207,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>29100</v>
       </c>
@@ -7226,7 +7230,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>45800</v>
       </c>
@@ -7249,7 +7253,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>54600</v>
       </c>
@@ -7272,7 +7276,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>55000</v>
       </c>
@@ -7295,7 +7299,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>56700</v>
       </c>
@@ -7318,7 +7322,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>60000</v>
       </c>

</xml_diff>